<commit_message>
added Modellraum line to Kosten_Prognose
</commit_message>
<xml_diff>
--- a/docs/Kosten_Prognose.xlsx
+++ b/docs/Kosten_Prognose.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCUser\Documents\Projekte\mini-climate-control\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\School\Diplomarbeit\SCC_2109\mini-climate-control\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32DF16BF-4B6E-4F56-901F-68830EB8BC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2459B54-6C0F-4E05-BB8F-5221601B7242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1073" yWindow="1073" windowWidth="21600" windowHeight="11872" xr2:uid="{9A33E93A-2FFC-4E05-A037-0ECCD8CDDAF5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A33E93A-2FFC-4E05-A037-0ECCD8CDDAF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>Kostenprognose Diplomarbeit SCC-2109</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Sensorplatine</t>
+  </si>
+  <si>
+    <t>Modellraum</t>
   </si>
 </sst>
 </file>
@@ -422,18 +425,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E167685E-88B8-427D-B1F2-3012ADA46F04}">
-  <dimension ref="B3:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B3:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>2</v>
       </c>
@@ -441,12 +444,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>